<commit_message>
Time series data update
</commit_message>
<xml_diff>
--- a/Time_series_data.xlsx
+++ b/Time_series_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64aae3e7249de19e/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64aae3e7249de19e/Documents/DATA309-Housing-Affordability/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{337E3E88-031D-4C18-A848-C403A45C26FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6824D946-1EDC-4004-9EE1-2325B2BCF9D5}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{337E3E88-031D-4C18-A848-C403A45C26FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94B8BB00-21B0-4497-8636-5EF38D0DF776}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>Mean NZ house price</t>
+  </si>
+  <si>
+    <t>Median Sale Price</t>
   </si>
 </sst>
 </file>
@@ -466,13 +469,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z142"/>
+  <dimension ref="A1:AA142"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="26" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -551,8 +554,11 @@
       <c r="Z1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>42005</v>
       </c>
@@ -595,8 +601,11 @@
       <c r="Z2" s="3">
         <v>402000</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA2">
+        <v>425000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>42036</v>
       </c>
@@ -639,8 +648,11 @@
       <c r="Z3" s="3">
         <v>410000</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA3">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>42064</v>
       </c>
@@ -717,8 +729,11 @@
       <c r="Z4" s="3">
         <v>415000</v>
       </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA4">
+        <v>475000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>42095</v>
       </c>
@@ -761,8 +776,11 @@
       <c r="Z5" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA5">
+        <v>455000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>42125</v>
       </c>
@@ -805,8 +823,11 @@
       <c r="Z6" s="3">
         <v>407000</v>
       </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA6">
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>42156</v>
       </c>
@@ -863,8 +884,11 @@
       <c r="Z7" s="3">
         <v>422000</v>
       </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA7">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>42186</v>
       </c>
@@ -907,8 +931,11 @@
       <c r="Z8" s="3">
         <v>420000</v>
       </c>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA8">
+        <v>464000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>42217</v>
       </c>
@@ -951,8 +978,11 @@
       <c r="Z9" s="3">
         <v>415000</v>
       </c>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA9">
+        <v>465000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>42248</v>
       </c>
@@ -1009,8 +1039,11 @@
       <c r="Z10" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA10">
+        <v>482000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>42278</v>
       </c>
@@ -1053,8 +1086,11 @@
       <c r="Z11" s="3">
         <v>421000</v>
       </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA11">
+        <v>458000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>42309</v>
       </c>
@@ -1097,8 +1133,11 @@
       <c r="Z12" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA12">
+        <v>457000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>42339</v>
       </c>
@@ -1155,8 +1194,11 @@
       <c r="Z13" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA13">
+        <v>462300</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>42370</v>
       </c>
@@ -1199,8 +1241,11 @@
       <c r="Z14" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA14">
+        <v>448000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>42401</v>
       </c>
@@ -1243,8 +1288,11 @@
       <c r="Z15" s="3">
         <v>424000</v>
       </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA15">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>42430</v>
       </c>
@@ -1323,8 +1371,11 @@
       <c r="Z16" s="3">
         <v>430000</v>
       </c>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA16">
+        <v>494000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>42461</v>
       </c>
@@ -1367,8 +1418,11 @@
       <c r="Z17" s="3">
         <v>430000</v>
       </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA17">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>42491</v>
       </c>
@@ -1411,8 +1465,11 @@
       <c r="Z18" s="3">
         <v>440000</v>
       </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA18">
+        <v>508000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>42522</v>
       </c>
@@ -1469,8 +1526,11 @@
       <c r="Z19" s="3">
         <v>431000</v>
       </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA19">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>42552</v>
       </c>
@@ -1513,8 +1573,11 @@
       <c r="Z20" s="3">
         <v>430000</v>
       </c>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA20">
+        <v>501000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>42583</v>
       </c>
@@ -1557,8 +1620,11 @@
       <c r="Z21" s="3">
         <v>422500</v>
       </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA21">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>42614</v>
       </c>
@@ -1615,8 +1681,11 @@
       <c r="Z22" s="3">
         <v>440000</v>
       </c>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA22">
+        <v>519000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>42644</v>
       </c>
@@ -1659,8 +1728,11 @@
       <c r="Z23" s="3">
         <v>430927</v>
       </c>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA23">
+        <v>510000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>42675</v>
       </c>
@@ -1703,8 +1775,11 @@
       <c r="Z24" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA24">
+        <v>520000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>42705</v>
       </c>
@@ -1761,8 +1836,11 @@
       <c r="Z25" s="3">
         <v>442000</v>
       </c>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA25">
+        <v>520000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>42736</v>
       </c>
@@ -1805,8 +1883,11 @@
       <c r="Z26" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA26">
+        <v>485500</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>42767</v>
       </c>
@@ -1849,8 +1930,11 @@
       <c r="Z27" s="3">
         <v>430000</v>
       </c>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA27">
+        <v>496000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>42795</v>
       </c>
@@ -1929,8 +2013,11 @@
       <c r="Z28" s="3">
         <v>449000</v>
       </c>
-    </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA28">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>42826</v>
       </c>
@@ -1973,8 +2060,11 @@
       <c r="Z29" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA29">
+        <v>540000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>42856</v>
       </c>
@@ -2017,8 +2107,11 @@
       <c r="Z30" s="3">
         <v>435000</v>
       </c>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA30">
+        <v>535000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>42887</v>
       </c>
@@ -2075,8 +2168,11 @@
       <c r="Z31" s="3">
         <v>435000</v>
       </c>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA31">
+        <v>530000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>42917</v>
       </c>
@@ -2119,8 +2215,11 @@
       <c r="Z32" s="3">
         <v>420000</v>
       </c>
-    </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA32">
+        <v>518000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>42948</v>
       </c>
@@ -2163,8 +2262,11 @@
       <c r="Z33" s="3">
         <v>427000</v>
       </c>
-    </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA33">
+        <v>530000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>42979</v>
       </c>
@@ -2221,8 +2323,11 @@
       <c r="Z34" s="3">
         <v>431500</v>
       </c>
-    </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA34">
+        <v>525000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>43009</v>
       </c>
@@ -2265,8 +2370,11 @@
       <c r="Z35" s="3">
         <v>450000</v>
       </c>
-    </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA35">
+        <v>530000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>43040</v>
       </c>
@@ -2309,8 +2417,11 @@
       <c r="Z36" s="3">
         <v>460000</v>
       </c>
-    </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA36">
+        <v>540000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>43070</v>
       </c>
@@ -2367,8 +2478,11 @@
       <c r="Z37" s="3">
         <v>435000</v>
       </c>
-    </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA37">
+        <v>551750</v>
+      </c>
+    </row>
+    <row r="38" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>43101</v>
       </c>
@@ -2411,8 +2525,11 @@
       <c r="Z38" s="3">
         <v>435000</v>
       </c>
-    </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA38">
+        <v>520000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>43132</v>
       </c>
@@ -2455,8 +2572,11 @@
       <c r="Z39" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA39">
+        <v>530000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>43160</v>
       </c>
@@ -2535,8 +2655,11 @@
       <c r="Z40" s="3">
         <v>450000</v>
       </c>
-    </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA40">
+        <v>560000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>43191</v>
       </c>
@@ -2579,8 +2702,11 @@
       <c r="Z41" s="3">
         <v>441000</v>
       </c>
-    </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA41">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>43221</v>
       </c>
@@ -2623,8 +2749,11 @@
       <c r="Z42" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA42">
+        <v>560000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>43252</v>
       </c>
@@ -2681,8 +2810,11 @@
       <c r="Z43" s="3">
         <v>432500</v>
       </c>
-    </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA43">
+        <v>560000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>43282</v>
       </c>
@@ -2725,8 +2857,11 @@
       <c r="Z44" s="3">
         <v>430000</v>
       </c>
-    </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA44">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>43313</v>
       </c>
@@ -2769,8 +2904,11 @@
       <c r="Z45" s="3">
         <v>425000</v>
       </c>
-    </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA45">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>43344</v>
       </c>
@@ -2827,8 +2965,11 @@
       <c r="Z46" s="3">
         <v>447500</v>
       </c>
-    </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA46">
+        <v>559000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>43374</v>
       </c>
@@ -2871,8 +3012,11 @@
       <c r="Z47" s="3">
         <v>465000</v>
       </c>
-    </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA47">
+        <v>561500</v>
+      </c>
+    </row>
+    <row r="48" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>43405</v>
       </c>
@@ -2915,8 +3059,11 @@
       <c r="Z48" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA48">
+        <v>580000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>43435</v>
       </c>
@@ -2973,8 +3120,11 @@
       <c r="Z49" s="3">
         <v>455000</v>
       </c>
-    </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA49">
+        <v>560000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>43466</v>
       </c>
@@ -3017,8 +3167,11 @@
       <c r="Z50" s="3">
         <v>430000</v>
       </c>
-    </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA50">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>43497</v>
       </c>
@@ -3061,8 +3214,11 @@
       <c r="Z51" s="3">
         <v>455000</v>
       </c>
-    </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA51">
+        <v>560000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>43525</v>
       </c>
@@ -3141,8 +3297,11 @@
       <c r="Z52" s="3">
         <v>459000</v>
       </c>
-    </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA52">
+        <v>585000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>43556</v>
       </c>
@@ -3185,8 +3344,11 @@
       <c r="Z53" s="3">
         <v>450000</v>
       </c>
-    </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA53">
+        <v>580000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>43586</v>
       </c>
@@ -3229,8 +3391,11 @@
       <c r="Z54" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA54">
+        <v>580000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>43617</v>
       </c>
@@ -3287,8 +3452,11 @@
       <c r="Z55" s="3">
         <v>445000</v>
       </c>
-    </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA55">
+        <v>585000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>43647</v>
       </c>
@@ -3331,8 +3499,11 @@
       <c r="Z56" s="3">
         <v>446000</v>
       </c>
-    </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA56">
+        <v>575000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>43678</v>
       </c>
@@ -3375,8 +3546,11 @@
       <c r="Z57" s="3">
         <v>440000</v>
       </c>
-    </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA57">
+        <v>580000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>43709</v>
       </c>
@@ -3433,8 +3607,11 @@
       <c r="Z58" s="3">
         <v>450000</v>
       </c>
-    </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA58">
+        <v>596956</v>
+      </c>
+    </row>
+    <row r="59" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>43739</v>
       </c>
@@ -3477,8 +3654,11 @@
       <c r="Z59" s="3">
         <v>465000</v>
       </c>
-    </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA59">
+        <v>605000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>43770</v>
       </c>
@@ -3521,8 +3701,11 @@
       <c r="Z60" s="3">
         <v>465000</v>
       </c>
-    </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA60">
+        <v>632000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>43800</v>
       </c>
@@ -3579,8 +3762,11 @@
       <c r="Z61" s="3">
         <v>460000</v>
       </c>
-    </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA61">
+        <v>628000</v>
+      </c>
+    </row>
+    <row r="62" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>43831</v>
       </c>
@@ -3623,8 +3809,11 @@
       <c r="Z62" s="3">
         <v>465000</v>
       </c>
-    </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA62">
+        <v>612000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>43862</v>
       </c>
@@ -3667,8 +3856,11 @@
       <c r="Z63" s="3">
         <v>474000</v>
       </c>
-    </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA63">
+        <v>635000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>43891</v>
       </c>
@@ -3747,8 +3939,11 @@
       <c r="Z64" s="3">
         <v>488000</v>
       </c>
-    </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA64">
+        <v>665000</v>
+      </c>
+    </row>
+    <row r="65" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>43922</v>
       </c>
@@ -3791,8 +3986,11 @@
       <c r="Z65" s="3">
         <v>464000</v>
       </c>
-    </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA65">
+        <v>680000</v>
+      </c>
+    </row>
+    <row r="66" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>43952</v>
       </c>
@@ -3835,8 +4033,11 @@
       <c r="Z66" s="3">
         <v>460000</v>
       </c>
-    </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA66">
+        <v>620000</v>
+      </c>
+    </row>
+    <row r="67" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>43983</v>
       </c>
@@ -3893,8 +4094,11 @@
       <c r="Z67" s="3">
         <v>470000</v>
       </c>
-    </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA67">
+        <v>637000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>44013</v>
       </c>
@@ -3937,8 +4141,11 @@
       <c r="Z68" s="3">
         <v>477000</v>
       </c>
-    </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA68">
+        <v>659500</v>
+      </c>
+    </row>
+    <row r="69" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>44044</v>
       </c>
@@ -3981,8 +4188,11 @@
       <c r="Z69" s="3">
         <v>498000</v>
       </c>
-    </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA69">
+        <v>677400</v>
+      </c>
+    </row>
+    <row r="70" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>44075</v>
       </c>
@@ -4039,8 +4249,11 @@
       <c r="Z70" s="3">
         <v>504000</v>
       </c>
-    </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA70">
+        <v>689000</v>
+      </c>
+    </row>
+    <row r="71" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>44105</v>
       </c>
@@ -4083,8 +4296,11 @@
       <c r="Z71" s="3">
         <v>510000</v>
       </c>
-    </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA71">
+        <v>725000</v>
+      </c>
+    </row>
+    <row r="72" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>44136</v>
       </c>
@@ -4127,8 +4343,11 @@
       <c r="Z72" s="3">
         <v>525000</v>
       </c>
-    </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA72">
+        <v>747000</v>
+      </c>
+    </row>
+    <row r="73" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>44166</v>
       </c>
@@ -4185,8 +4404,11 @@
       <c r="Z73" s="3">
         <v>540000</v>
       </c>
-    </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA73">
+        <v>745000</v>
+      </c>
+    </row>
+    <row r="74" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>44197</v>
       </c>
@@ -4229,8 +4451,11 @@
       <c r="Z74" s="3">
         <v>507500</v>
       </c>
-    </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA74">
+        <v>730300</v>
+      </c>
+    </row>
+    <row r="75" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>44228</v>
       </c>
@@ -4273,8 +4498,11 @@
       <c r="Z75" s="3">
         <v>560000</v>
       </c>
-    </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA75">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>44256</v>
       </c>
@@ -4353,8 +4581,11 @@
       <c r="Z76" s="3">
         <v>575000</v>
       </c>
-    </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA76">
+        <v>825000</v>
+      </c>
+    </row>
+    <row r="77" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>44287</v>
       </c>
@@ -4397,8 +4628,11 @@
       <c r="Z77" s="3">
         <v>566000</v>
       </c>
-    </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA77">
+        <v>804362</v>
+      </c>
+    </row>
+    <row r="78" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>44317</v>
       </c>
@@ -4441,8 +4675,11 @@
       <c r="Z78" s="3">
         <v>580000</v>
       </c>
-    </row>
-    <row r="79" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA78">
+        <v>820000</v>
+      </c>
+    </row>
+    <row r="79" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>44348</v>
       </c>
@@ -4499,8 +4736,11 @@
       <c r="Z79" s="3">
         <v>565000</v>
       </c>
-    </row>
-    <row r="80" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA79">
+        <v>816000</v>
+      </c>
+    </row>
+    <row r="80" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>44378</v>
       </c>
@@ -4543,8 +4783,11 @@
       <c r="Z80" s="3">
         <v>597000</v>
       </c>
-    </row>
-    <row r="81" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA80">
+        <v>825000</v>
+      </c>
+    </row>
+    <row r="81" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>44409</v>
       </c>
@@ -4587,8 +4830,11 @@
       <c r="Z81" s="3">
         <v>620000</v>
       </c>
-    </row>
-    <row r="82" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA81">
+        <v>850000</v>
+      </c>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>44440</v>
       </c>
@@ -4645,8 +4891,11 @@
       <c r="Z82" s="3">
         <v>657500</v>
       </c>
-    </row>
-    <row r="83" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA82">
+        <v>795000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>44470</v>
       </c>
@@ -4689,8 +4938,11 @@
       <c r="Z83" s="3">
         <v>665000</v>
       </c>
-    </row>
-    <row r="84" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA83">
+        <v>892000</v>
+      </c>
+    </row>
+    <row r="84" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>44501</v>
       </c>
@@ -4733,8 +4985,11 @@
       <c r="Z84" s="3">
         <v>690000</v>
       </c>
-    </row>
-    <row r="85" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA84">
+        <v>925000</v>
+      </c>
+    </row>
+    <row r="85" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>44531</v>
       </c>
@@ -4791,8 +5046,11 @@
       <c r="Z85" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="86" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA85">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="86" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>44562</v>
       </c>
@@ -4835,8 +5093,11 @@
       <c r="Z86" s="3">
         <v>650000</v>
       </c>
-    </row>
-    <row r="87" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA86">
+        <v>879000</v>
+      </c>
+    </row>
+    <row r="87" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>44593</v>
       </c>
@@ -4879,8 +5140,11 @@
       <c r="Z87" s="3">
         <v>717830</v>
       </c>
-    </row>
-    <row r="88" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA87">
+        <v>885000</v>
+      </c>
+    </row>
+    <row r="88" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>44621</v>
       </c>
@@ -4959,8 +5223,11 @@
       <c r="Z88" s="3">
         <v>700000</v>
       </c>
-    </row>
-    <row r="89" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA88">
+        <v>890000</v>
+      </c>
+    </row>
+    <row r="89" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>44652</v>
       </c>
@@ -5003,8 +5270,11 @@
       <c r="Z89" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="90" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA89">
+        <v>875000</v>
+      </c>
+    </row>
+    <row r="90" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>44682</v>
       </c>
@@ -5047,8 +5317,11 @@
       <c r="Z90" s="3">
         <v>687000</v>
       </c>
-    </row>
-    <row r="91" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA90">
+        <v>850000</v>
+      </c>
+    </row>
+    <row r="91" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>44713</v>
       </c>
@@ -5105,8 +5378,11 @@
       <c r="Z91" s="3">
         <v>685000</v>
       </c>
-    </row>
-    <row r="92" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA91">
+        <v>850000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>44743</v>
       </c>
@@ -5149,8 +5425,11 @@
       <c r="Z92" s="3">
         <v>675000</v>
       </c>
-    </row>
-    <row r="93" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA92">
+        <v>810000</v>
+      </c>
+    </row>
+    <row r="93" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>44774</v>
       </c>
@@ -5193,8 +5472,11 @@
       <c r="Z93" s="3">
         <v>650000</v>
       </c>
-    </row>
-    <row r="94" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA93">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="94" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>44805</v>
       </c>
@@ -5251,8 +5533,11 @@
       <c r="Z94" s="3">
         <v>675000</v>
       </c>
-    </row>
-    <row r="95" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA94">
+        <v>810000</v>
+      </c>
+    </row>
+    <row r="95" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>44835</v>
       </c>
@@ -5295,8 +5580,11 @@
       <c r="Z95" s="3">
         <v>659000</v>
       </c>
-    </row>
-    <row r="96" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA95">
+        <v>818000</v>
+      </c>
+    </row>
+    <row r="96" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>44866</v>
       </c>
@@ -5339,8 +5627,11 @@
       <c r="Z96" s="3">
         <v>665000</v>
       </c>
-    </row>
-    <row r="97" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA96">
+        <v>806000</v>
+      </c>
+    </row>
+    <row r="97" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>44896</v>
       </c>
@@ -5397,8 +5688,11 @@
       <c r="Z97" s="3">
         <v>651000</v>
       </c>
-    </row>
-    <row r="98" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA97">
+        <v>785000</v>
+      </c>
+    </row>
+    <row r="98" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>44927</v>
       </c>
@@ -5441,8 +5735,11 @@
       <c r="Z98" s="3">
         <v>642500</v>
       </c>
-    </row>
-    <row r="99" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA98">
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="99" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>44958</v>
       </c>
@@ -5485,8 +5782,11 @@
       <c r="Z99" s="3">
         <v>670000</v>
       </c>
-    </row>
-    <row r="100" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA99">
+        <v>766000</v>
+      </c>
+    </row>
+    <row r="100" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>44986</v>
       </c>
@@ -5565,8 +5865,11 @@
       <c r="Z100" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="101" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA100">
+        <v>779000</v>
+      </c>
+    </row>
+    <row r="101" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>45017</v>
       </c>
@@ -5609,8 +5912,11 @@
       <c r="Z101" s="3">
         <v>665000</v>
       </c>
-    </row>
-    <row r="102" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA101">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="102" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>45047</v>
       </c>
@@ -5653,8 +5959,11 @@
       <c r="Z102" s="3">
         <v>649000</v>
       </c>
-    </row>
-    <row r="103" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA102">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="103" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>45078</v>
       </c>
@@ -5711,8 +6020,11 @@
       <c r="Z103" s="3">
         <v>657000</v>
       </c>
-    </row>
-    <row r="104" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA103">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="104" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>45108</v>
       </c>
@@ -5755,8 +6067,11 @@
       <c r="Z104" s="3">
         <v>665000</v>
       </c>
-    </row>
-    <row r="105" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA104">
+        <v>770000</v>
+      </c>
+    </row>
+    <row r="105" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>45139</v>
       </c>
@@ -5799,8 +6114,11 @@
       <c r="Z105" s="3">
         <v>659000</v>
       </c>
-    </row>
-    <row r="106" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA105">
+        <v>770000</v>
+      </c>
+    </row>
+    <row r="106" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>45170</v>
       </c>
@@ -5857,8 +6175,11 @@
       <c r="Z106" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="107" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA106">
+        <v>799000</v>
+      </c>
+    </row>
+    <row r="107" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>45200</v>
       </c>
@@ -5901,8 +6222,11 @@
       <c r="Z107" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="108" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA107">
+        <v>789500</v>
+      </c>
+    </row>
+    <row r="108" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>45231</v>
       </c>
@@ -5945,8 +6269,11 @@
       <c r="Z108" s="3">
         <v>700000</v>
       </c>
-    </row>
-    <row r="109" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA108">
+        <v>795000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A109" s="2">
         <v>45261</v>
       </c>
@@ -6003,8 +6330,11 @@
       <c r="Z109" s="3">
         <v>665000</v>
       </c>
-    </row>
-    <row r="110" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA109">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="110" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>45292</v>
       </c>
@@ -6047,8 +6377,11 @@
       <c r="Z110" s="3">
         <v>646000</v>
       </c>
-    </row>
-    <row r="111" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA110">
+        <v>763000</v>
+      </c>
+    </row>
+    <row r="111" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
         <v>45323</v>
       </c>
@@ -6091,8 +6424,11 @@
       <c r="Z111" s="3">
         <v>705000</v>
       </c>
-    </row>
-    <row r="112" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA111">
+        <v>791000</v>
+      </c>
+    </row>
+    <row r="112" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>45352</v>
       </c>
@@ -6171,8 +6507,11 @@
       <c r="Z112" s="3">
         <v>695000</v>
       </c>
-    </row>
-    <row r="113" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA112">
+        <v>801000</v>
+      </c>
+    </row>
+    <row r="113" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>45383</v>
       </c>
@@ -6215,8 +6554,11 @@
       <c r="Z113" s="3">
         <v>670000</v>
       </c>
-    </row>
-    <row r="114" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA113">
+        <v>790000</v>
+      </c>
+    </row>
+    <row r="114" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>45413</v>
       </c>
@@ -6259,8 +6601,11 @@
       <c r="Z114" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="115" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA114">
+        <v>770000</v>
+      </c>
+    </row>
+    <row r="115" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>45444</v>
       </c>
@@ -6317,8 +6662,11 @@
       <c r="Z115" s="3">
         <v>690000</v>
       </c>
-    </row>
-    <row r="116" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA115">
+        <v>770000</v>
+      </c>
+    </row>
+    <row r="116" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A116" s="2">
         <v>45474</v>
       </c>
@@ -6361,8 +6709,11 @@
       <c r="Z116" s="3">
         <v>650500</v>
       </c>
-    </row>
-    <row r="117" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA116">
+        <v>754000</v>
+      </c>
+    </row>
+    <row r="117" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>45505</v>
       </c>
@@ -6405,8 +6756,11 @@
       <c r="Z117" s="3">
         <v>662500</v>
       </c>
-    </row>
-    <row r="118" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA117">
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="118" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>45536</v>
       </c>
@@ -6463,8 +6817,11 @@
       <c r="Z118" s="3">
         <v>690000</v>
       </c>
-    </row>
-    <row r="119" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA118">
+        <v>782000</v>
+      </c>
+    </row>
+    <row r="119" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>45566</v>
       </c>
@@ -6507,8 +6864,11 @@
       <c r="Z119" s="3">
         <v>700000</v>
       </c>
-    </row>
-    <row r="120" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA119">
+        <v>795000</v>
+      </c>
+    </row>
+    <row r="120" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>45597</v>
       </c>
@@ -6551,8 +6911,11 @@
       <c r="Z120" s="3">
         <v>699000</v>
       </c>
-    </row>
-    <row r="121" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA120">
+        <v>790000</v>
+      </c>
+    </row>
+    <row r="121" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>45627</v>
       </c>
@@ -6609,8 +6972,11 @@
       <c r="Z121" s="3">
         <v>700000</v>
       </c>
-    </row>
-    <row r="122" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA121">
+        <v>776000</v>
+      </c>
+    </row>
+    <row r="122" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>45658</v>
       </c>
@@ -6653,8 +7019,11 @@
       <c r="Z122" s="3">
         <v>677000</v>
       </c>
-    </row>
-    <row r="123" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA122">
+        <v>750000</v>
+      </c>
+    </row>
+    <row r="123" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>45689</v>
       </c>
@@ -6697,8 +7066,11 @@
       <c r="Z123" s="3">
         <v>705000</v>
       </c>
-    </row>
-    <row r="124" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA123">
+        <v>770000</v>
+      </c>
+    </row>
+    <row r="124" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>45717</v>
       </c>
@@ -6775,8 +7147,11 @@
       <c r="Z124" s="3">
         <v>690000</v>
       </c>
-    </row>
-    <row r="125" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA124">
+        <v>790000</v>
+      </c>
+    </row>
+    <row r="125" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>45748</v>
       </c>
@@ -6819,8 +7194,11 @@
       <c r="Z125" s="3">
         <v>695652</v>
       </c>
-    </row>
-    <row r="126" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA125">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="126" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>45778</v>
       </c>
@@ -6863,8 +7241,11 @@
       <c r="Z126" s="3">
         <v>680000</v>
       </c>
-    </row>
-    <row r="127" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA126">
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="127" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>45809</v>
       </c>
@@ -6919,8 +7300,11 @@
       <c r="Z127" s="3">
         <v>675000</v>
       </c>
-    </row>
-    <row r="128" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA127">
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="128" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>45839</v>
       </c>
@@ -6963,8 +7347,11 @@
       <c r="Z128" s="3">
         <v>677000</v>
       </c>
-    </row>
-    <row r="129" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA128">
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="129" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>45870</v>
       </c>
@@ -7007,8 +7394,11 @@
       <c r="Z129" s="3">
         <v>690000</v>
       </c>
-    </row>
-    <row r="130" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA129">
+        <v>760000</v>
+      </c>
+    </row>
+    <row r="130" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>45901</v>
       </c>
@@ -7063,8 +7453,11 @@
       <c r="Z130" s="3">
         <v>709000</v>
       </c>
-    </row>
-    <row r="131" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA130">
+        <v>773000</v>
+      </c>
+    </row>
+    <row r="131" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>45931</v>
       </c>
@@ -7107,8 +7500,11 @@
       <c r="Z131" s="3">
         <v>708000</v>
       </c>
-    </row>
-    <row r="132" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA131">
+        <v>790000</v>
+      </c>
+    </row>
+    <row r="132" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>45962</v>
       </c>
@@ -7151,8 +7547,11 @@
       <c r="Z132" s="3">
         <v>725000</v>
       </c>
-    </row>
-    <row r="133" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA132">
+        <v>802000</v>
+      </c>
+    </row>
+    <row r="133" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>45992</v>
       </c>
@@ -7207,8 +7606,11 @@
       <c r="Z133" s="3">
         <v>721000</v>
       </c>
-    </row>
-    <row r="134" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA133">
+        <v>790000</v>
+      </c>
+    </row>
+    <row r="134" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>46023</v>
       </c>
@@ -7251,8 +7653,11 @@
       <c r="Z134" s="3">
         <v>700000</v>
       </c>
-    </row>
-    <row r="135" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA134">
+        <v>755000</v>
+      </c>
+    </row>
+    <row r="135" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>46054</v>
       </c>
@@ -7289,8 +7694,11 @@
       <c r="Z135" s="3">
         <v>719000</v>
       </c>
-    </row>
-    <row r="136" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA135">
+        <v>795000</v>
+      </c>
+    </row>
+    <row r="136" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>46082</v>
       </c>
@@ -7349,8 +7757,11 @@
       <c r="Z136" s="3">
         <v>715000</v>
       </c>
-    </row>
-    <row r="137" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA136">
+        <v>790000</v>
+      </c>
+    </row>
+    <row r="137" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A137" s="2">
         <v>46113</v>
       </c>
@@ -7387,8 +7798,11 @@
       <c r="Z137" s="3">
         <v>705000</v>
       </c>
-    </row>
-    <row r="138" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA137">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="138" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>46143</v>
       </c>
@@ -7425,8 +7839,11 @@
       <c r="Z138" s="3">
         <v>725000</v>
       </c>
-    </row>
-    <row r="139" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA138">
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="139" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>46174</v>
       </c>
@@ -7467,8 +7884,11 @@
       <c r="Z139" s="3">
         <v>710000</v>
       </c>
-    </row>
-    <row r="140" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA139">
+        <v>775000</v>
+      </c>
+    </row>
+    <row r="140" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>46204</v>
       </c>
@@ -7503,8 +7923,11 @@
         <v>296.10165360000002</v>
       </c>
       <c r="Z140" s="3"/>
-    </row>
-    <row r="141" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA140">
+        <v>760500</v>
+      </c>
+    </row>
+    <row r="141" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>46235</v>
       </c>
@@ -7537,8 +7960,11 @@
         <v>300.83523769999999</v>
       </c>
       <c r="Z141" s="3"/>
-    </row>
-    <row r="142" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA141">
+        <v>750000</v>
+      </c>
+    </row>
+    <row r="142" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>46266</v>
       </c>

</xml_diff>